<commit_message>
x_day_earlier: Friday Wisconsin via Wisconsin Coach Lines O'Hare 07:30 -> Kenosha 08:15, back 08:45 -> O'Hare 09:30 (Nick)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_day_earlier.xlsx
+++ b/docs/x_day_earlier.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1736,37 +1736,42 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>11:50</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>35th &amp; State St (Four Winds shuttle)</t>
+          <t>O'Hare Multi-Modal Facility (CTA Red from 95th, Blue to O'Hare, airport train)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri 14:30 ET</t>
+          <t>Fri 08:15</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Kenosha Brat Stop (WI)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Four Winds Casino Shuttle (Chinatown)</t>
+          <t>Wisconsin Coach Lines</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Chinatown 11:50 CT -&gt; Four Winds New Buffalo 14:30 ET</t>
+          <t>Wisconsin Coach O'Hare -&gt; Kenosha -&gt; Milwaukee</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Sat Nov 21</t>
+          <t>(Metra)</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Wisconsin: replaces Metra UP-N (weekday schedule). Back on the 08:45 south.</t>
         </is>
       </c>
     </row>
@@ -1783,37 +1788,42 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Kenosha Brat Stop</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fri 18:55</t>
+          <t>Fri 09:30</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+          <t>O'Hare (then Blue + Red to Sox-35th, ~10:40)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Four Winds Casino Shuttle (Chinatown)</t>
+          <t>Wisconsin Coach Lines</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Four Winds New Buffalo 18:30 ET (site prints 17:30) -&gt; Chinatown 18:55 CT (arrival assumed)</t>
+          <t>Wisconsin Coach Milwaukee -&gt; Kenosha -&gt; O'Hare</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Sat Nov 21</t>
+          <t>(Metra)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Four Winds shuttle 11:50 from 35th &amp; State. If the 07:30 is missed, the 09:30 north works only with a later shuttle.</t>
         </is>
       </c>
     </row>
@@ -1830,32 +1840,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>35th &amp; State St (Four Winds shuttle)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sat 06:00</t>
+          <t>Fri 14:30 ET</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Jefferson Lines</t>
+          <t>Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>JL Chicago 21:15 -&gt; Davenport -&gt; Iowa City -&gt; Des Moines -&gt; Omaha 06:00 (daily assumed)</t>
+          <t>Chinatown 11:50 CT -&gt; Four Winds New Buffalo 14:30 ET</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1867,114 +1877,208 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>day 11</t>
+          <t>day 10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Fri 18:55</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Four Winds Casino Shuttle (Chinatown)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Four Winds New Buffalo 18:30 ET (site prints 17:30) -&gt; Chinatown 18:55 CT (arrival assumed)</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>Sat Nov 21</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>06:15</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Omaha</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Sat 09:45</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Sioux Falls</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Jefferson Lines</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>JL Omaha 06:15 -&gt; Sioux City -&gt; Vermillion -&gt; Sioux Falls 09:45 (intermediate times assumed; daily assumed)</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Sun Nov 22</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sat 06:00</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>JL Chicago 21:15 -&gt; Davenport -&gt; Iowa City -&gt; Des Moines -&gt; Omaha 06:00 (daily assumed)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sat Nov 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>day 11</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Sat Nov 21</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sat 09:45</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>JL Omaha 06:15 -&gt; Sioux City -&gt; Vermillion -&gt; Sioux Falls 09:45 (intermediate times assumed; daily assumed)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Sun Nov 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>day 11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Sat Nov 21</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Sioux Falls</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Sat 14:05</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Fargo</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Jefferson Lines</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>JL Sioux Falls 10:00 -&gt; Brookings -&gt; Watertown -&gt; Summit Corner -&gt; Sisseton Jct -&gt; Fargo 14:05 (daily assumed)</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Sun Nov 22</t>
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Kenosha by Metra is not in the booked sheet (walk-up). Booked Sat Nov 21 06:32 -&gt; 08:15, back 09:08 -&gt; 10:50; a day earlier it is Fri Nov 20 on the weekday UP-N schedule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Finish: Fargo arrives Sat Nov 21 14:05 a day earlier, so MATBUS runs (Saturday): Route 17 / Route 4 into Moorhead, or the walk.</t>
-        </is>
-      </c>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" t="inlineStr">
+        <is>
+          <t>Kenosha: Wisconsin Coach Lines from O'Hare (rows above), not Metra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Finish: Fargo arrives Sat Nov 21 14:05 a day earlier, so MATBUS runs (Saturday): Route 17 / Route 4 into Moorhead, or the walk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Every other ride runs at the same times the day before (checked in the timetable data); confirm on the carrier sites as for the booking.</t>
         </is>

</xml_diff>

<commit_message>
x_day_earlier: Friday Wisconsin plan A Hiawatha Chicago 06:10 -> Milwaukee 07:49, back 08:05 -> 09:44 (Nick); Wisconsin Coach via O'Hare as plan B
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/x_day_earlier.xlsx
+++ b/docs/x_day_earlier.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,11 @@
         <fgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,11 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1736,32 +1742,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>06:10</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>O'Hare Multi-Modal Facility (CTA Red from 95th, Blue to O'Hare, airport train)</t>
+          <t>Chicago Union Station (CTA Red 95th -&gt; Jackson, walk; ~15 min margin)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fri 08:15</t>
+          <t>Fri 07:49</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Kenosha Brat Stop (WI)</t>
+          <t>Milwaukee (WI)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Wisconsin Coach Lines</t>
+          <t>Amtrak</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Wisconsin Coach O'Hare -&gt; Kenosha -&gt; Milwaukee</t>
+          <t>Hiawatha</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1771,7 +1777,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Wisconsin: replaces Metra UP-N (weekday schedule). Back on the 08:45 south.</t>
+          <t>Wisconsin, plan A: Hiawatha up and back (Nick).</t>
         </is>
       </c>
     </row>
@@ -1788,136 +1794,146 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>08:05</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Fri 09:44</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Chicago Union Station (then Red to Sox-35th)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Amtrak</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Hiawatha</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>(Metra)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Four Winds 11:50 from 35th &amp; State. Plan B below: Wisconsin Coach via O'Hare if the 06:10 is missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>O'Hare Multi-Modal Facility (CTA Red from 95th, Blue to O'Hare, airport train)</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Fri 08:15</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Kenosha Brat Stop (WI)</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Wisconsin Coach Lines</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Wisconsin Coach O'Hare -&gt; Kenosha -&gt; Milwaukee</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>(Metra)</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Plan B (if the 06:10 Hiawatha is missed): Wisconsin: replaces Metra UP-N (weekday schedule). Back on the 08:45 south.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Kenosha Brat Stop</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Fri 09:30</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>O'Hare (then Blue + Red to Sox-35th, ~10:40)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>Wisconsin Coach Lines</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Wisconsin Coach Milwaukee -&gt; Kenosha -&gt; O'Hare</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>(Metra)</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Four Winds shuttle 11:50 from 35th &amp; State. If the 07:30 is missed, the 09:30 north works only with a later shuttle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>day 10</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Fri Nov 20</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>11:50</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>35th &amp; State St (Four Winds shuttle)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Fri 14:30 ET</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Four Winds Casino Shuttle (Chinatown)</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Chinatown 11:50 CT -&gt; Four Winds New Buffalo 14:30 ET</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Sat Nov 21</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>day 10</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Fri Nov 20</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Fri 18:55</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Four Winds Casino Shuttle (Chinatown)</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Four Winds New Buffalo 18:30 ET (site prints 17:30) -&gt; Chinatown 18:55 CT (arrival assumed)</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Sat Nov 21</t>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Plan B (if the 06:10 Hiawatha is missed): Four Winds shuttle 11:50 from 35th &amp; State. If the 07:30 is missed, the 09:30 north works only with a later shuttle.</t>
         </is>
       </c>
     </row>
@@ -1934,32 +1950,32 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>35th &amp; State St (Four Winds shuttle)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Sat 06:00</t>
+          <t>Fri 14:30 ET</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Jefferson Lines</t>
+          <t>Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>JL Chicago 21:15 -&gt; Davenport -&gt; Iowa City -&gt; Des Moines -&gt; Omaha 06:00 (daily assumed)</t>
+          <t>Chinatown 11:50 CT -&gt; Four Winds New Buffalo 14:30 ET</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1971,114 +1987,208 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>day 11</t>
+          <t>day 10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fri 18:55</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Four Winds Casino Shuttle (Chinatown)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Four Winds New Buffalo 18:30 ET (site prints 17:30) -&gt; Chinatown 18:55 CT (arrival assumed)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>Sat Nov 21</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>06:15</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Omaha</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Sat 09:45</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Sioux Falls</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Jefferson Lines</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>JL Omaha 06:15 -&gt; Sioux City -&gt; Vermillion -&gt; Sioux Falls 09:45 (intermediate times assumed; daily assumed)</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Sun Nov 22</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>day 10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sat 06:00</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>JL Chicago 21:15 -&gt; Davenport -&gt; Iowa City -&gt; Des Moines -&gt; Omaha 06:00 (daily assumed)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sat Nov 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>day 11</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Sat Nov 21</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sat 09:45</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>JL Omaha 06:15 -&gt; Sioux City -&gt; Vermillion -&gt; Sioux Falls 09:45 (intermediate times assumed; daily assumed)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Sun Nov 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>day 11</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sat Nov 21</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Sioux Falls</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Sat 14:05</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Fargo</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Jefferson Lines</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>JL Sioux Falls 10:00 -&gt; Brookings -&gt; Watertown -&gt; Summit Corner -&gt; Sisseton Jct -&gt; Fargo 14:05 (daily assumed)</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Sun Nov 22</t>
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Kenosha: Wisconsin Coach Lines from O'Hare (rows above), not Metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Finish: Fargo arrives Sat Nov 21 14:05 a day earlier, so MATBUS runs (Saturday): Route 17 / Route 4 into Moorhead, or the walk.</t>
-        </is>
-      </c>
-    </row>
+    <row r="37"/>
     <row r="38">
       <c r="B38" t="inlineStr">
+        <is>
+          <t>Kenosha: Wisconsin Coach Lines from O'Hare (rows above), not Metra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Finish: Fargo arrives Sat Nov 21 14:05 a day earlier, so MATBUS runs (Saturday): Route 17 / Route 4 into Moorhead, or the walk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Every other ride runs at the same times the day before (checked in the timetable data); confirm on the carrier sites as for the booking.</t>
         </is>

</xml_diff>